<commit_message>
Add import mode selector, employee-ID device linking, drop DOB from template
- ImportPanel: three import modes (Employees & devices / Employees only /
  Devices only) filter recognized sheets before validation — a file with
  both sheets can now be imported partially without touching the other side
- Devices sheet: new Employee ID column links a device to its owner by
  exact ID match, with "Assigned To" (name/e-mail/username) as a fuzzy
  fallback when ID isn't given — ID matching is more reliable for partial
  data than name matching
- Employees sheet: removed the Date of Birth column/field, per request
- Regenerated import-template.xlsx to match (DOB column dropped, Employee
  ID column added to Devices, with column widths for readability)
</commit_message>
<xml_diff>
--- a/square-frontend/public/import-template.xlsx
+++ b/square-frontend/public/import-template.xlsx
@@ -398,7 +398,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="7.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -426,12 +438,9 @@
         <v>Emergency Contact</v>
       </c>
       <c r="I1" t="str">
-        <v>Date of Birth</v>
+        <v>Location</v>
       </c>
       <c r="J1" t="str">
-        <v>Location</v>
-      </c>
-      <c r="K1" t="str">
         <v>Floor</v>
       </c>
     </row>
@@ -461,12 +470,9 @@
         <v>+8801811223344</v>
       </c>
       <c r="I2" t="str">
-        <v>1995-06-15</v>
+        <v>Anita Center (HQ)</v>
       </c>
       <c r="J2" t="str">
-        <v>Anita Center (HQ)</v>
-      </c>
-      <c r="K2" t="str">
         <v>4</v>
       </c>
     </row>
@@ -496,25 +502,38 @@
         <v>+8801811223345</v>
       </c>
       <c r="I3" t="str">
-        <v>1997-01-20</v>
+        <v>Sector 3 Office</v>
       </c>
       <c r="J3" t="str">
-        <v>Sector 3 Office</v>
-      </c>
-      <c r="K3" t="str">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="32.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -548,12 +567,15 @@
         <v>Assigned To</v>
       </c>
       <c r="K1" t="str">
+        <v>Employee ID</v>
+      </c>
+      <c r="L1" t="str">
         <v>Department</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>IP Address</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Specifications</v>
       </c>
     </row>
@@ -589,18 +611,21 @@
         <v/>
       </c>
       <c r="K2" t="str">
+        <v>SQ-EMP-0999</v>
+      </c>
+      <c r="L2" t="str">
         <v>Commercial</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>10.20.4.201</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>Core i7 · 16GB RAM · 512GB NVMe</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add employee promotion — quick action, bulk CSV import, distinct audit trail
Superuser can now promote an employee directly from All Employees (a
focused designation-only action alongside the existing full Manage
flow), or bulk-promote via a new "Promotions" import mode: match by
Employee ID, resolve issues through the same AI-chat flow as other
imports, and enforce one-unique-designation-per-department both
against the current roster and within the file itself.

Designation changes are now logged as EMPLOYEE_PROMOTED (old → new)
in the audit trail, distinct from a generic PROFILE_UPDATED.
</commit_message>
<xml_diff>
--- a/square-frontend/public/import-template.xlsx
+++ b/square-frontend/public/import-template.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="Employees" sheetId="1" r:id="rId1"/>
     <sheet name="Devices" sheetId="2" r:id="rId2"/>
+    <sheet name="Promotions" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -399,19 +400,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K3"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="7.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -528,22 +516,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N2"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
-    <col min="13" max="13" width="16.83203125" customWidth="1"/>
-    <col min="14" max="14" width="32.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -638,4 +610,70 @@
     <ignoredError numberStoredAsText="1" sqref="A1:N2"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G2"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="17.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Employee ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>New Designation</v>
+      </c>
+      <c r="D1" t="str">
+        <v>New Department</v>
+      </c>
+      <c r="E1" t="str">
+        <v>New Unit</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Effective Date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>EMP-0001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Jane Doe</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Senior Officer</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>